<commit_message>
Excel file sai uuendatud
</commit_message>
<xml_diff>
--- a/TextPad 7/TextPad_Test_Report_and_Bug_report_template.xlsx
+++ b/TextPad 7/TextPad_Test_Report_and_Bug_report_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\opilane\source\repos\HenryKuningas\TarkvarasysteemideTestimine\TextPad 7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B844F9E7-B5AD-4863-923B-92806B79698C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02E8FA7-C723-4375-9084-1313068E3CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16410" yWindow="8535" windowWidth="23925" windowHeight="12315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11490" yWindow="7080" windowWidth="23925" windowHeight="12315" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Report" sheetId="11" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="53">
   <si>
     <t>Product:</t>
   </si>
@@ -204,31 +204,49 @@
     <t>Truncation 'Browse…' in 'Manage files' dialog</t>
   </si>
   <si>
+    <t>Truncation 'Bering Information' in 'About TextPad' dialog</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>4, 5</t>
+  </si>
+  <si>
+    <t>7, 8, 9, 10</t>
+  </si>
+  <si>
+    <t>11, 12</t>
+  </si>
+  <si>
+    <t>1, 2, 3</t>
+  </si>
+  <si>
     <t>Steps to reproduce: 
 1. Launch 'TextPad'
 2. Go to 'Help' -&gt; 'About TextPad'
 Expected result:
-There are no truncations
+There are no truncation
 Actual result: 
 There are truncations</t>
   </si>
   <si>
-    <t>Truncation 'Bering Information' in 'About TextPad' dialog</t>
-  </si>
-  <si>
-    <t>1, 2</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>4, 5</t>
-  </si>
-  <si>
-    <t>7, 8, 9, 10</t>
-  </si>
-  <si>
-    <t>11, 12</t>
+    <t>1.	Launch TextPad
+2.	Open any document containing text data
+3.	Go to File -&gt; Print… to invoke Print dialog 
+Expected result:
+There are no truncations
+Actual result:
+There are truncations</t>
+  </si>
+  <si>
+    <t>1.	Launch TextPad
+2.	Open any document containing text data
+3.	Go to File -&gt; Print… to invoke Print dialog 
+Expected result:
+There are no misalignments present
+Actual result:
+There are misalignments present</t>
   </si>
 </sst>
 </file>
@@ -1068,10 +1086,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Pilt 1">
+        <xdr:cNvPr id="3" name="Pilt 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0D89428-AAB7-4082-B818-A22E2AEDE127}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB9AEA2F-4E0B-4848-8ABA-C9A3BBAB46C1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1697,10 +1715,10 @@
         <v>21</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D2" s="34" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1711,10 +1729,10 @@
         <v>21</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D3" s="35" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1738,7 +1756,7 @@
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="33" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1760,7 +1778,7 @@
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="35" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4193,7 +4211,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="180.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4201,7 +4219,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="228.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4274,7 +4292,9 @@
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="32" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="9" spans="2:3" ht="243" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="7" t="s">
@@ -4284,7 +4304,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4346,7 +4367,9 @@
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="32" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="9" spans="2:3" ht="241.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="7" t="s">
@@ -4577,6 +4600,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBDF2EF6028720478E3F27B9B31ABD09" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af4c30ee4a8bd4ac003a3d536b29f91a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="615ccdff-0541-46ac-a88f-a8d1251c2b60" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c50b0a04c06fbcee891037f18b70482d" ns2:_="">
     <xsd:import namespace="615ccdff-0541-46ac-a88f-a8d1251c2b60"/>
@@ -4716,22 +4754,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C53E4B81-85CB-4814-992F-9FCD036E17F1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20789A9-57E9-4886-B95B-F2A34AEE83F1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="615ccdff-0541-46ac-a88f-a8d1251c2b60"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C37B6576-FA83-4FDB-AFBB-5436182600AB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4747,28 +4794,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20789A9-57E9-4886-B95B-F2A34AEE83F1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="615ccdff-0541-46ac-a88f-a8d1251c2b60"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C53E4B81-85CB-4814-992F-9FCD036E17F1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>